<commit_message>
selesai menggenarate kalimat menjadi 7000 lebih
</commit_message>
<xml_diff>
--- a/ABSA_db_kalimat_komentar.xlsx
+++ b/ABSA_db_kalimat_komentar.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\sentimen-absa\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44BC7DDD-74FD-48B9-B23F-3DE818B24273}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{956EE64F-71F2-45D2-86C1-00963BAD6B84}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" xr2:uid="{359AE8BC-56C0-4424-B3FB-77FA9BFC594B}"/>
   </bookViews>
@@ -2676,13 +2676,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58136DF1-DCB1-451F-BC4B-942EDA03FCCC}">
-  <dimension ref="A1:D1617"/>
+  <dimension ref="A1:E1617"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="33.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="99.85546875" style="5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="29" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="87.5703125" style="5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -23069,7 +23070,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="1457" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1457" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1457" s="2">
         <v>1456</v>
       </c>
@@ -23083,7 +23084,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="1458" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1458" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1458" s="2">
         <v>1457</v>
       </c>
@@ -23096,8 +23097,12 @@
       <c r="D1458" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1459" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1458" s="5" t="str">
+        <f>_xlfn.CONCAT(C1458,".")</f>
+        <v>sehat selalu nak pondok laksana uji thobaqoh tahap iii ujian tulis selenggara februari.</v>
+      </c>
+    </row>
+    <row r="1459" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1459" s="2">
         <v>1458</v>
       </c>
@@ -23110,8 +23115,12 @@
       <c r="D1459" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1460" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1459" s="5" t="str">
+        <f t="shared" ref="E1459:E1522" si="0">_xlfn.CONCAT(C1459,".")</f>
+        <v>masya allah laksana thobaqoh tahap iii ujian tulis selenggara februari.</v>
+      </c>
+    </row>
+    <row r="1460" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1460" s="2">
         <v>1459</v>
       </c>
@@ -23124,8 +23133,12 @@
       <c r="D1460" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1461" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1460" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>moga uji thobaqoh tahap iii uji tulis selenggara dilaksanakan pada bulan februari.</v>
+      </c>
+    </row>
+    <row r="1461" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1461" s="2">
         <v>1460</v>
       </c>
@@ -23138,8 +23151,12 @@
       <c r="D1461" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1462" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1461" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>anak azkiyah kamila laksana uji thobaqoh di ihya ulumuddin tahap iii uji tulis selenggara pada bulan februari.</v>
+      </c>
+    </row>
+    <row r="1462" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1462" s="2">
         <v>1461</v>
       </c>
@@ -23152,8 +23169,12 @@
       <c r="D1462" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1463" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1462" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>: moga lancar ujianx anak aidy arun arifah temanx yang lain aamiin laksana ujian thobaqoh ihya ulumuddin tahap iii uji tulis selenggara februari.</v>
+      </c>
+    </row>
+    <row r="1463" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1463" s="2">
         <v>1462</v>
       </c>
@@ -23166,8 +23187,12 @@
       <c r="D1463" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1464" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1463" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>aamiin semogah jalan lancar menyelenggarakan uji thobaqoh tahap iii pada uji tulis selenggara pada bulan februari.</v>
+      </c>
+    </row>
+    <row r="1464" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1464" s="2">
         <v>1463</v>
       </c>
@@ -23180,8 +23205,12 @@
       <c r="D1464" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1465" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1464" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>aamiin xd semangat anak laksana uji thobaqoh nurzahra alya nabila askar tahap iii uji tulis selenggara februari.</v>
+      </c>
+    </row>
+    <row r="1465" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1465" s="2">
         <v>1464</v>
       </c>
@@ -23194,8 +23223,12 @@
       <c r="D1465" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1466" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1465" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>moga uji anak mudah dan dapat hasil yang baik laksana uji thobaqoh di ihya ulumuddin tahap iii pada uji tulis selenggara februari.</v>
+      </c>
+    </row>
+    <row r="1466" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1466" s="2">
         <v>1465</v>
       </c>
@@ -23208,8 +23241,12 @@
       <c r="D1466" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1467" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1466" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>moga semua lancar uji anak laksana uji thobaqoh tahap iii ujian tulis selenggara februari.</v>
+      </c>
+    </row>
+    <row r="1467" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1467" s="2">
         <v>1466</v>
       </c>
@@ -23222,8 +23259,12 @@
       <c r="D1467" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1468" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="E1467" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>: moga ujianx lancar mudah laksana uji thobaqoh tahap iii ujian tulis selenggara februari.</v>
+      </c>
+    </row>
+    <row r="1468" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A1468" s="2">
         <v>1467</v>
       </c>
@@ -23236,8 +23277,12 @@
       <c r="D1468" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1469" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1468" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Bismillahirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahman.</v>
+      </c>
+    </row>
+    <row r="1469" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1469" s="2">
         <v>1468</v>
       </c>
@@ -23250,8 +23295,12 @@
       <c r="D1469" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1470" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1469" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>aamiin... ...laksana uji thobaqoh tahap iii ujian tulis selenggara februari.</v>
+      </c>
+    </row>
+    <row r="1470" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1470" s="2">
         <v>1469</v>
       </c>
@@ -23264,8 +23313,12 @@
       <c r="D1470" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1471" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1470" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>assalamualaikum bu ustazah, saya mau tanya tanggal berapa pulangnya para Santriwati informasi izinnya sudah ditutup..</v>
+      </c>
+    </row>
+    <row r="1471" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1471" s="2">
         <v>1470</v>
       </c>
@@ -23278,8 +23331,12 @@
       <c r="D1471" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1472" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1471" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>kuliah harus cepat libur kalau ingin pulang bantu orang tua cari duit bagang kurang abk kodong bagang informasi izin pondok ditutup.</v>
+      </c>
+    </row>
+    <row r="1472" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1472" s="2">
         <v>1471</v>
       </c>
@@ -23292,8 +23349,12 @@
       <c r="D1472" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1473" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1472" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>klu anak sakit bagaimana apa nda pulang informasi izin pondok ditutup.</v>
+      </c>
+    </row>
+    <row r="1473" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1473" s="2">
         <v>1472</v>
       </c>
@@ -23306,8 +23367,12 @@
       <c r="D1473" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1474" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1473" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Semoga anak-anak selalu sehat dan selamat dalam informasi izin pondokan ditutup.</v>
+      </c>
+    </row>
+    <row r="1474" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1474" s="2">
         <v>1473</v>
       </c>
@@ -23320,8 +23385,12 @@
       <c r="D1474" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1475" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="E1474" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Hari raya cinta ibu korban kuat ibu terimah kasih semua ibu telah beri cinta perhati korban batas selamat hari ibu.</v>
+      </c>
+    </row>
+    <row r="1475" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A1475" s="2">
         <v>1474</v>
       </c>
@@ -23334,8 +23403,12 @@
       <c r="D1475" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1476" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1475" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>hari kita raya cinta korban kuat ibu terimah kasih semua ibu telah beri cinta perhati korban batas selamat hari ibu hari kita raya cinta korban kuat ibu terimah kasih semua ibu telah beri cinta perhati korban batas selamat hari ibu.</v>
+      </c>
+    </row>
+    <row r="1476" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1476" s="2">
         <v>1475</v>
       </c>
@@ -23348,8 +23421,12 @@
       <c r="D1476" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1477" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1476" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Selamat Hari Ibu Dunia Hari Kita Raya Cinta Korban Kuat Ibu Terimah kasih ibu semua telah memberi cinta korban batas.</v>
+      </c>
+    </row>
+    <row r="1477" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1477" s="2">
         <v>1476</v>
       </c>
@@ -23362,8 +23439,12 @@
       <c r="D1477" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1478" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1477" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Selamat Hari Ibu, Hari Raya Cinta Ibu Korban Kuat Ibu Terimah kasih semua ibu telah memberi cinta perhati.</v>
+      </c>
+    </row>
+    <row r="1478" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1478" s="2">
         <v>1477</v>
       </c>
@@ -23376,8 +23457,12 @@
       <c r="D1478" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1479" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="E1478" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>masya allah hari kita raya cinta ibu korban kuat ibu terima kasih semua ibu telah memberi cinta perhati korban batas selamat hari ibu.</v>
+      </c>
+    </row>
+    <row r="1479" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A1479" s="2">
         <v>1478</v>
       </c>
@@ -23390,8 +23475,12 @@
       <c r="D1479" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1480" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1479" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Terima kasih anak-anak yang cantik, semoga amal ibadahnya tetap terjaga, jagalah pondok agar tetap lindungi allah swt hari kita raya cinta korban kuat ibu terimah kasih semua ibu telah beri cinta perhati korban batas selamat hari ibu.</v>
+      </c>
+    </row>
+    <row r="1480" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1480" s="2">
         <v>1479</v>
       </c>
@@ -23404,8 +23493,12 @@
       <c r="D1480" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1481" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1480" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Selamat Hari Guru Guru Besar Indonesia Kuat.</v>
+      </c>
+    </row>
+    <row r="1481" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1481" s="2">
         <v>1480</v>
       </c>
@@ -23418,8 +23511,12 @@
       <c r="D1481" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1482" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1481" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Terima kasih ustzah cantik selalu mendampingi anak mulai bangun tidur lelap dalam menuntut ilmu selamat hari guru guru hebat Indonesia kuat.</v>
+      </c>
+    </row>
+    <row r="1482" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1482" s="2">
         <v>1481</v>
       </c>
@@ -23432,8 +23529,12 @@
       <c r="D1482" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1483" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1482" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Sehat sll ustzh selamat hari guru guru hebat Indonesia kuat.</v>
+      </c>
+    </row>
+    <row r="1483" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1483" s="2">
         <v>1482</v>
       </c>
@@ -23446,8 +23547,12 @@
       <c r="D1483" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1484" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1483" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Selamat Hari Guru, semoga sehat selalu, guru hebat Indonesia kuat.</v>
+      </c>
+    </row>
+    <row r="1484" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1484" s="2">
         <v>1483</v>
       </c>
@@ -23460,8 +23565,12 @@
       <c r="D1484" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1485" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1484" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Terima kasih ustadz senang bisa mendampingi anak dalam menuntut ilmu selamat hari guru sehat selalu selamat hari guru guru hebat Indonesia kuat.</v>
+      </c>
+    </row>
+    <row r="1485" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1485" s="2">
         <v>1484</v>
       </c>
@@ -23474,8 +23583,12 @@
       <c r="D1485" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1486" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1485" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Selamat Hari Guru Ustadzd Ustadzda Selamat Hari Guru Guru Besar Indonesia Kuat.</v>
+      </c>
+    </row>
+    <row r="1486" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1486" s="2">
         <v>1485</v>
       </c>
@@ -23488,8 +23601,12 @@
       <c r="D1486" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1487" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1486" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Selamat Hari Guru, terima kasih, bimbing anak kami sehat, semangat, berkah, setiap orang, Selamat Hari Guru, guru hebat Indonesia kuat.</v>
+      </c>
+    </row>
+    <row r="1487" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1487" s="2">
         <v>1486</v>
       </c>
@@ -23502,8 +23619,12 @@
       <c r="D1487" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1488" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1487" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Selamat Hari Guru Nasional Selamat Hari Guru Guru Besar Indonesia Kuat.</v>
+      </c>
+    </row>
+    <row r="1488" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1488" s="2">
         <v>1487</v>
       </c>
@@ -23516,8 +23637,12 @@
       <c r="D1488" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1489" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1488" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Selamat Hari Guru Guru Besar Indonesia Kuat.</v>
+      </c>
+    </row>
+    <row r="1489" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1489" s="2">
         <v>1488</v>
       </c>
@@ -23530,8 +23655,12 @@
       <c r="D1489" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1490" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1489" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>happy teacher day selamat hari guru guru hebat Indonesia kuat.</v>
+      </c>
+    </row>
+    <row r="1490" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1490" s="2">
         <v>1489</v>
       </c>
@@ -23544,8 +23673,12 @@
       <c r="D1490" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1491" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1490" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Alhamdulillah moga anak anakku lulus tobaqoh lanjut lebih tingkat yang blum lulus lebih giat lagi ajar moga uji tahap ikut lulus galeri umum hasil uji thobaqoh tahap ii.</v>
+      </c>
+    </row>
+    <row r="1491" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1491" s="2">
         <v>1490</v>
       </c>
@@ -23558,8 +23691,12 @@
       <c r="D1491" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1492" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1491" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Masya Allah, semoga anak-anak lulus galeri umum hasil uji thobaqoh tahap ii di ihya ulumiddin putri.</v>
+      </c>
+    </row>
+    <row r="1492" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1492" s="2">
         <v>1491</v>
       </c>
@@ -23572,8 +23709,12 @@
       <c r="D1492" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1493" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1492" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>masya allah galeri umum hasil uji thobaqoh tahap ii di ihya ulumiddin putri.</v>
+      </c>
+    </row>
+    <row r="1493" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1493" s="2">
         <v>1492</v>
       </c>
@@ -23586,12 +23727,16 @@
       <c r="D1493" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1494" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1493" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>xd smoga putri q naik ke kitab slnjutnya aamiiin xd trims tak t hingga ustadzah snntiasa m bimbing anak galeri umum hasil uji thobaqoh tahap ii.</v>
+      </c>
+    </row>
+    <row r="1494" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1494" s="2">
         <v>1493</v>
       </c>
-      <c r="B1494" s="7" t="s">
+      <c r="B1494" s="8" t="s">
         <v>745</v>
       </c>
       <c r="C1494" s="4" t="s">
@@ -23600,8 +23745,12 @@
       <c r="D1494" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1495" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1494" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>masyaallah xd moga lulus semua ana allah galeri umum hasil uji thobaqoh tahap ii ihya ulumiddin putri.</v>
+      </c>
+    </row>
+    <row r="1495" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1495" s="2">
         <v>1494</v>
       </c>
@@ -23614,8 +23763,12 @@
       <c r="D1495" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1496" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1495" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>masya allah moga lulus kasi anak galeri umum hasil uji thobaqoh tahap ii di ihya ulumiddin putri.</v>
+      </c>
+    </row>
+    <row r="1496" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1496" s="2">
         <v>1495</v>
       </c>
@@ -23628,8 +23781,12 @@
       <c r="D1496" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1497" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1496" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>alhamdulillah galeri umum hasil uji thobaqoh tahap ii ihya ulumiddin putri.</v>
+      </c>
+    </row>
+    <row r="1497" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1497" s="2">
         <v>1496</v>
       </c>
@@ -23642,8 +23799,12 @@
       <c r="D1497" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1498" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1497" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>aamiin galeri umum hasil uji thobaqoh tahap ii di ihya ulumiddin putri.</v>
+      </c>
+    </row>
+    <row r="1498" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1498" s="2">
         <v>1497</v>
       </c>
@@ -23656,8 +23817,12 @@
       <c r="D1498" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1499" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1498" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>amiin galeri umum hasil uji thobaqoh tahap ii di ihya ulumiddin putri.</v>
+      </c>
+    </row>
+    <row r="1499" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1499" s="2">
         <v>1498</v>
       </c>
@@ -23670,8 +23835,12 @@
       <c r="D1499" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1500" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1499" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>moga anak lulus galeri umum hasil uji thobaqoh tahap ii di ihya ulumiddin putri.</v>
+      </c>
+    </row>
+    <row r="1500" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1500" s="2">
         <v>1499</v>
       </c>
@@ -23684,8 +23853,12 @@
       <c r="D1500" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1501" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1500" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>aamiin aamiin galeri umum hasil uji thobaqoh tahap ii di ihya ulumiddin putri.</v>
+      </c>
+    </row>
+    <row r="1501" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1501" s="2">
         <v>1500</v>
       </c>
@@ -23698,8 +23871,12 @@
       <c r="D1501" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1502" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1501" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>senang melihat anak lulus, terimakasih semua bimbing anak di pondok xd maaf ustadz mungkin dilampirkan kelulusan yang lulus di grup wa wali murid terima kasih belum galeri umum hasil uji thobaqoh tahap ii.</v>
+      </c>
+    </row>
+    <row r="1502" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1502" s="2">
         <v>1501</v>
       </c>
@@ -23712,8 +23889,12 @@
       <c r="D1502" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1503" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1502" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>alhamdulillah galeri umum hasil uji thobaqoh tahap ii ihya ulumiddin putri.</v>
+      </c>
+    </row>
+    <row r="1503" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1503" s="2">
         <v>1502</v>
       </c>
@@ -23726,8 +23907,12 @@
       <c r="D1503" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1504" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1503" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>semuga pondok serta keluarga besar pondok selalu diberkahi allah selalu mendapat berkah dari rosulullah nabi muhammad s a w galeri umum hasil uji thobaqoh tahap ii di ihya ulumiddin putri.</v>
+      </c>
+    </row>
+    <row r="1504" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1504" s="2">
         <v>1503</v>
       </c>
@@ -23740,8 +23925,12 @@
       <c r="D1504" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1505" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1504" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>allah moga anak mudah menjawab soal beri hari uji alih thobaqoh tahap ii ihya ulumiddin.</v>
+      </c>
+    </row>
+    <row r="1505" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1505" s="2">
         <v>1504</v>
       </c>
@@ -23754,8 +23943,12 @@
       <c r="D1505" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1506" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1505" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>masya allah hari uji alih tahap ii thobaqoh di ihya ulumiddin.</v>
+      </c>
+    </row>
+    <row r="1506" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1506" s="2">
         <v>1505</v>
       </c>
@@ -23768,8 +23961,12 @@
       <c r="D1506" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1507" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1506" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>allah mudah untk menjawab soal uji anak aamiin hari uji alih thobaqoh tahap ii ihya ulumiddin.</v>
+      </c>
+    </row>
+    <row r="1507" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1507" s="2">
         <v>1506</v>
       </c>
@@ -23782,8 +23979,12 @@
       <c r="D1507" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1508" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1507" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>masya allah hari uji alih tahap ii thobaqoh di ihya ulumiddin.</v>
+      </c>
+    </row>
+    <row r="1508" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1508" s="2">
         <v>1507</v>
       </c>
@@ -23796,8 +23997,12 @@
       <c r="D1508" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1509" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1508" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Semangat anakku hari uji alih thobaqoh tahap ii di ihya ulumiddin.</v>
+      </c>
+    </row>
+    <row r="1509" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1509" s="2">
         <v>1508</v>
       </c>
@@ -23810,8 +24015,12 @@
       <c r="D1509" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1510" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1509" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Tetap semangat nak hari laksana uji alih thobaqoh tahap ii uji lisan mulai thobaqoh tajwid fathul muin.</v>
+      </c>
+    </row>
+    <row r="1510" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1510" s="2">
         <v>1509</v>
       </c>
@@ -23824,8 +24033,12 @@
       <c r="D1510" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1511" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1510" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>bismillah, moga allah mudah lancar, uji lisan alih thobaqoh tahap ii, uji lisan mulai thobaqoh tajwid fathul muin.</v>
+      </c>
+    </row>
+    <row r="1511" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1511" s="2">
         <v>1510</v>
       </c>
@@ -23838,8 +24051,12 @@
       <c r="D1511" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1512" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1511" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>bismillah mudah anak hari laksana uji alih thobaqoh tahap ii uji lisan mulai thobaqoh tajwid fathul muin.</v>
+      </c>
+    </row>
+    <row r="1512" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1512" s="2">
         <v>1511</v>
       </c>
@@ -23852,8 +24069,12 @@
       <c r="D1512" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1513" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1512" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Semangat q semua nak, insya allah mudah lancar uji lisannya hari laksana uji alih thobaqoh tahap ii uji lisan mulai thobaqoh tajwid fathul muin.</v>
+      </c>
+    </row>
+    <row r="1513" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1513" s="2">
         <v>1512</v>
       </c>
@@ -23866,8 +24087,12 @@
       <c r="D1513" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1514" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1513" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>bismillah moga lancar semua nak hari laksana uji alih thobaqoh tahap ii uji lisan mulai thobaqoh tajwid fathul muin.</v>
+      </c>
+    </row>
+    <row r="1514" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1514" s="2">
         <v>1513</v>
       </c>
@@ -23880,8 +24105,12 @@
       <c r="D1514" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1515" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1514" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>bismillah allah mudah an anak jawab semua amin hari laksana uji alih thobaqoh tahap ii uji lisan mulai thobaqoh tajwid fathul muin.</v>
+      </c>
+    </row>
+    <row r="1515" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1515" s="2">
         <v>1514</v>
       </c>
@@ -23894,8 +24123,12 @@
       <c r="D1515" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1516" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="E1515" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>masya allah moga dmudahkan nak hari laksana uji alih thobaqoh tahap ii uji lisan mulai thobaqoh tajwid fathul muin.</v>
+      </c>
+    </row>
+    <row r="1516" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A1516" s="2">
         <v>1515</v>
       </c>
@@ -23908,8 +24141,12 @@
       <c r="D1516" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1517" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1516" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Bismillahirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahmanirrahman.</v>
+      </c>
+    </row>
+    <row r="1517" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1517" s="2">
         <v>1516</v>
       </c>
@@ -23922,8 +24159,12 @@
       <c r="D1517" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1518" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1517" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>moga lancar uji hari laksana uji alih thobaqoh tahap ii uji lisan mulai thobaqoh tajwid fathul muin.</v>
+      </c>
+    </row>
+    <row r="1518" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1518" s="2">
         <v>1517</v>
       </c>
@@ -23936,8 +24177,12 @@
       <c r="D1518" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1519" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="E1518" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>mama sini berMotivasi/Spiritual semoga hari laksana uji alih thobaqoh tahap ii uji lisan mulai thobaqoh tajwid fathul muin.</v>
+      </c>
+    </row>
+    <row r="1519" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A1519" s="2">
         <v>1518</v>
       </c>
@@ -23950,8 +24195,12 @@
       <c r="D1519" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1520" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1519" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>assalamualaikum xd dar masuk ustadzah mungkin hasil uji anak kirim grup wa wali murid wali murid wali murid wali murid utama pribadi ustadzah penasaran hasil uji anak xd syukron ustadzah uji alih thobaqoh tahap ii ihya ulumiddin uji tulis.</v>
+      </c>
+    </row>
+    <row r="1520" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1520" s="2">
         <v>1519</v>
       </c>
@@ -23964,8 +24213,12 @@
       <c r="D1520" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1521" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1520" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>moga mudah semua uji tobaqoh anak sholehaku aaaaaamin uji alih thobaqoh tahap ii ihya ulumiddin uji tulis.</v>
+      </c>
+    </row>
+    <row r="1521" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1521" s="2">
         <v>1520</v>
       </c>
@@ -23978,8 +24231,12 @@
       <c r="D1521" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1522" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1521" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>: maasyaallah uji coba alih thobaqoh tahap ii di ihya ulumiddin uji tulis.</v>
+      </c>
+    </row>
+    <row r="1522" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1522" s="2">
         <v>1521</v>
       </c>
@@ -23992,8 +24249,12 @@
       <c r="D1522" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1523" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1522" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>uji alih thobaqoh tahap ii ihya ulumiddin uji tulis.</v>
+      </c>
+    </row>
+    <row r="1523" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1523" s="2">
         <v>1522</v>
       </c>
@@ -24006,8 +24267,12 @@
       <c r="D1523" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1524" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1523" s="5" t="str">
+        <f t="shared" ref="E1523:E1586" si="1">_xlfn.CONCAT(C1523,".")</f>
+        <v>masyaallah moga semuax lancar uji alih thobaqoh tahap ii ihya ulumiddin uji tulis.</v>
+      </c>
+    </row>
+    <row r="1524" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1524" s="2">
         <v>1523</v>
       </c>
@@ -24020,8 +24285,12 @@
       <c r="D1524" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1525" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1524" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>masya allah anak shaliha ademm melihat uji alih thobaqoh tahap ii ihya ulumiddin uji tulis.</v>
+      </c>
+    </row>
+    <row r="1525" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1525" s="2">
         <v>1524</v>
       </c>
@@ -24034,8 +24303,12 @@
       <c r="D1525" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1526" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1525" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>aaaaamin uji alih thobaqoh tahap ii ihya ulumiddin uji tulis.</v>
+      </c>
+    </row>
+    <row r="1526" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1526" s="2">
         <v>1525</v>
       </c>
@@ -24048,8 +24321,12 @@
       <c r="D1526" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1527" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1526" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>allah mudah semua uji tobaqoh anak-anak ppap utama dua putri sholehaku allah laksana uji alih thobaqoh tahap ii.</v>
+      </c>
+    </row>
+    <row r="1527" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1527" s="2">
         <v>1526</v>
       </c>
@@ -24062,8 +24339,12 @@
       <c r="D1527" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1528" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1527" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>aamiin laksana uji alih thobaqoh tahap ii,.</v>
+      </c>
+    </row>
+    <row r="1528" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1528" s="2">
         <v>1527</v>
       </c>
@@ -24076,8 +24357,12 @@
       <c r="D1528" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1529" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1528" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>allah moga semua siswa n alumni lolos tobaqo dan terus naik utama putri aamiin allah laksana uji alih thobaqoh tahap ii.</v>
+      </c>
+    </row>
+    <row r="1529" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1529" s="2">
         <v>1528</v>
       </c>
@@ -24090,8 +24375,12 @@
       <c r="D1529" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1530" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1529" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>amiin laksana uji alih thobaqoh tahap ii.</v>
+      </c>
+    </row>
+    <row r="1530" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1530" s="2">
         <v>1529</v>
       </c>
@@ -24104,8 +24393,12 @@
       <c r="D1530" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1531" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1530" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>allah mudah n lancar uji di hadap para siswa ppsp khusus putra n putriku aamiin yra laksana uji alih thobaqoh tahap ii.</v>
+      </c>
+    </row>
+    <row r="1531" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1531" s="2">
         <v>1530</v>
       </c>
@@ -24118,8 +24411,12 @@
       <c r="D1531" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1532" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1531" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>aamiiiin allah laksana uji coba alih thobaqoh tahap ii.</v>
+      </c>
+    </row>
+    <row r="1532" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1532" s="2">
         <v>1531</v>
       </c>
@@ -24132,8 +24429,12 @@
       <c r="D1532" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1533" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1532" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>Allah mudah anak anak dalam hadap uji laksana uji alih thobaqoh tahap ii.</v>
+      </c>
+    </row>
+    <row r="1533" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1533" s="2">
         <v>1532</v>
       </c>
@@ -24146,8 +24447,12 @@
       <c r="D1533" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1534" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1533" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>amin yarabbal alamin laksana uji alih thobaqoh tahap ii.</v>
+      </c>
+    </row>
+    <row r="1534" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1534" s="2">
         <v>1533</v>
       </c>
@@ -24160,8 +24465,12 @@
       <c r="D1534" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1535" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1534" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>aamiiin yaalllah laksana uji coba alih thobaqoh tahap ii.</v>
+      </c>
+    </row>
+    <row r="1535" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1535" s="2">
         <v>1534</v>
       </c>
@@ -24174,8 +24483,12 @@
       <c r="D1535" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1536" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1535" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>allomma sholli ala muhammad waala ali muhammad moga berkah salawat anak sholeh mudah tunduk uji muas sebentar akan laksana uji perampasan thobaqoh tahap ii tanggal november.</v>
+      </c>
+    </row>
+    <row r="1536" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1536" s="2">
         <v>1535</v>
       </c>
@@ -24188,8 +24501,12 @@
       <c r="D1536" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1537" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1536" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>smg semua siswa diberi kemudahan dalam hadap-hadapan sebentar akan menyelenggarakan uji coba thobaqoh tahap ii pada tanggal november.</v>
+      </c>
+    </row>
+    <row r="1537" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1537" s="2">
         <v>1536</v>
       </c>
@@ -24202,8 +24519,12 @@
       <c r="D1537" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1538" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1537" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>Alhamdulillah, mudah-mudahan, ikut uji Allah sebentar akan laksana uji coba thobaqoh tahap ii pada bulan november,.</v>
+      </c>
+    </row>
+    <row r="1538" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1538" s="2">
         <v>1537</v>
       </c>
@@ -24216,8 +24537,12 @@
       <c r="D1538" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1539" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1538" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>bismillah moga uji coba anak sebentar akan laksana uji coba thobaqoh tahap ii pada bulan november,.</v>
+      </c>
+    </row>
+    <row r="1539" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1539" s="2">
         <v>1538</v>
       </c>
@@ -24230,8 +24555,12 @@
       <c r="D1539" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1540" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1539" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>alhamdulillah anak dstu akan laksana sebentar uji coba thobaqoh tahap ii tanggal november:.</v>
+      </c>
+    </row>
+    <row r="1540" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1540" s="2">
         <v>1539</v>
       </c>
@@ -24244,8 +24573,12 @@
       <c r="D1540" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1541" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1540" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>aamiin sebentar akan laksana uji coba thobaqoh tahap ii pada tanggal november,.</v>
+      </c>
+    </row>
+    <row r="1541" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1541" s="2">
         <v>1540</v>
       </c>
@@ -24258,8 +24591,12 @@
       <c r="D1541" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1542" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1541" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>aamiin semoga anak-anak lulus semua aamiin salam orang tua wali astik ayu ananta pasangkayu sebentar lagi akan menyelenggarakan uji coba thobaqoh tahap ii pada tanggal november.</v>
+      </c>
+    </row>
+    <row r="1542" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1542" s="2">
         <v>1541</v>
       </c>
@@ -24272,8 +24609,12 @@
       <c r="D1542" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1543" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1542" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>moga anak-anak lulus semua aamiin yra sebentar akan menyelenggarakan uji coba thobaqoh tahap ii pada tanggal november.</v>
+      </c>
+    </row>
+    <row r="1543" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1543" s="2">
         <v>1542</v>
       </c>
@@ -24286,8 +24627,12 @@
       <c r="D1543" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1544" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1543" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>Mudah-mudahan usaha anak dalam uji sukses semua aamiin sebentar akan laksana uji coba ketidakberesan thobaqoh tahap ii pada november.</v>
+      </c>
+    </row>
+    <row r="1544" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1544" s="2">
         <v>1543</v>
       </c>
@@ -24300,8 +24645,12 @@
       <c r="D1544" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1545" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1544" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>allah akan laksana uji coba ketidakberesan thobaqoh tahap ii pada bulan november.</v>
+      </c>
+    </row>
+    <row r="1545" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1545" s="2">
         <v>1544</v>
       </c>
@@ -24314,8 +24663,12 @@
       <c r="D1545" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1546" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1545" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>bismillah rohmanirrohim moga semua ajar nya lulus dalam uji coba tahap ii, aamiin xd putri solehahku sebentar lagi akan menyelenggarakan uji coba thobaqoh tahap ii,.</v>
+      </c>
+    </row>
+    <row r="1546" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1546" s="2">
         <v>1545</v>
       </c>
@@ -24328,8 +24681,12 @@
       <c r="D1546" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1547" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1546" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>bismillah semoga ujian anak lulus aamiinn sebentar akan laksana uji coba thobaqoh tahap ii pada bulan november.</v>
+      </c>
+    </row>
+    <row r="1547" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1547" s="2">
         <v>1546</v>
       </c>
@@ -24342,8 +24699,12 @@
       <c r="D1547" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1548" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1547" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>amiin akan laksana pada uji coba thobaqoh tahap ii pada tanggal november.</v>
+      </c>
+    </row>
+    <row r="1548" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1548" s="2">
         <v>1547</v>
       </c>
@@ -24356,8 +24717,12 @@
       <c r="D1548" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1549" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1548" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>moga semua anak aaaaaamin mudah lulus ikut uji tobaqoh utama anak aaaaamin sebentar akan laksana uji coba peralahan thobaqoh tahap ii pada november.</v>
+      </c>
+    </row>
+    <row r="1549" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1549" s="2">
         <v>1548</v>
       </c>
@@ -24370,8 +24735,12 @@
       <c r="D1549" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1550" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1549" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>: moga mudah semua usaha anak anak Santri di uji semua amin amin wali Santri Nizaska Cha Manding sebentar akan menyelenggarakan uji coba thobaqoh tahap ii pada tanggal november,.</v>
+      </c>
+    </row>
+    <row r="1550" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1550" s="2">
         <v>1549</v>
       </c>
@@ -24384,8 +24753,12 @@
       <c r="D1550" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1551" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1550" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>moga semua murid mudah melakukan uji coba singkat akan laksana uji coba thobaqoh tahap ii pada tanggal november.</v>
+      </c>
+    </row>
+    <row r="1551" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1551" s="2">
         <v>1550</v>
       </c>
@@ -24398,8 +24771,12 @@
       <c r="D1551" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1552" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1551" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>Semogah anak lolos tahap lanjut salam mambi sebentar laksana uji coba thobaqoh tahap ii tanggal november.</v>
+      </c>
+    </row>
+    <row r="1552" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1552" s="2">
         <v>1551</v>
       </c>
@@ -24412,8 +24789,12 @@
       <c r="D1552" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1553" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1552" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>moga semua murid mudah melakukan uji coba singkat akan laksana uji coba thobaqoh tahap ii pada tanggal november.</v>
+      </c>
+    </row>
+    <row r="1553" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1553" s="2">
         <v>1552</v>
       </c>
@@ -24426,8 +24807,12 @@
       <c r="D1553" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1554" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1553" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>moga uji thobaqohnya mudah semua allah akan laksana uji coba peralahan thobaqoh tahap ii pada november.</v>
+      </c>
+    </row>
+    <row r="1554" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1554" s="2">
         <v>1553</v>
       </c>
@@ -24440,8 +24825,12 @@
       <c r="D1554" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1555" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1554" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>moga para alumni mudah melakukan uji sebut sebentar akan laksana uji coba thobaqoh tahap ii pada tanggal november.</v>
+      </c>
+    </row>
+    <row r="1555" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1555" s="2">
         <v>1554</v>
       </c>
@@ -24454,8 +24843,12 @@
       <c r="D1555" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1556" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1555" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>bismillah, moga ujianx lancar, naik tingkat selanjutx akan laksana uji coba thobaqoh tahap ii pada tanggal november,.</v>
+      </c>
+    </row>
+    <row r="1556" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1556" s="2">
         <v>1555</v>
       </c>
@@ -24468,8 +24861,12 @@
       <c r="D1556" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1557" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1556" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>bismillah, mudah mudahan anak anak mudah di ajar mudah mudahan lulus semua sebentar akan laksana uji coba thobaqoh tahap ii pada tanggal november.</v>
+      </c>
+    </row>
+    <row r="1557" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1557" s="2">
         <v>1556</v>
       </c>
@@ -24482,8 +24879,12 @@
       <c r="D1557" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1558" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1557" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>Mudah-mudahan anak-anak soleh hadap uji thobaqoh aamiinn moga ana lulus sebentar akan menyelenggarakan uji coba peralahan thobaqoh tahap ii tanggal november.</v>
+      </c>
+    </row>
+    <row r="1558" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1558" s="2">
         <v>1557</v>
       </c>
@@ -24496,8 +24897,12 @@
       <c r="D1558" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1559" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1558" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>allah lancar mudah allah sebentar akan laksana uji coba thobaqoh tahap ii tanggal november.</v>
+      </c>
+    </row>
+    <row r="1559" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1559" s="2">
         <v>1558</v>
       </c>
@@ -24510,8 +24915,12 @@
       <c r="D1559" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1560" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1559" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>moga anak-anak mudah menguji Allah sebentar akan laksana uji coba thobaqoh tahap ii pada november.</v>
+      </c>
+    </row>
+    <row r="1560" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1560" s="2">
         <v>1559</v>
       </c>
@@ -24524,8 +24933,12 @@
       <c r="D1560" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1561" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1560" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>bismillahirrahmanirrahim mudah han ana lulus dalam uji amin yra sebentar akan laksana uji coba thobaqoh tahap ii pada november.</v>
+      </c>
+    </row>
+    <row r="1561" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1561" s="2">
         <v>1560</v>
       </c>
@@ -24538,8 +24951,12 @@
       <c r="D1561" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1562" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1561" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>Selamat pagi pemuda, ingat hari sumpah pemuda oktober, maju bersama Indonesia Raya.</v>
+      </c>
+    </row>
+    <row r="1562" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1562" s="2">
         <v>1561</v>
       </c>
@@ -24552,8 +24969,12 @@
       <c r="D1562" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1563" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1562" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>Selamat Hari Santri untuk semua anak, semoga sukses selalu, lindungi allah subhanahu wataalah, selamat Hari Santri Nasional.</v>
+      </c>
+    </row>
+    <row r="1563" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1563" s="2">
         <v>1562</v>
       </c>
@@ -24566,8 +24987,12 @@
       <c r="D1563" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1564" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1563" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>Banyak pembullyan ponpes banyak siswa kabur xd siswa kabur hukum tampa tahu apa yang menyebabkan orang kabur ponpes pondok salafiyah parappe putri ada kegiatan sosialisasi tema cegah tangan keras satu.</v>
+      </c>
+    </row>
+    <row r="1564" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1564" s="2">
         <v>1563</v>
       </c>
@@ -24580,8 +25005,12 @@
       <c r="D1564" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1565" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1564" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>rindu adikq dstu pondok salafiyah parappe putri ada kegiatan sosialisasi tema cegah tangan keras satu didik.</v>
+      </c>
+    </row>
+    <row r="1565" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1565" s="2">
         <v>1564</v>
       </c>
@@ -24594,8 +25023,12 @@
       <c r="D1565" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1566" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1565" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>: mntp spy aman pondok tdk terlalu beri ganjar tdk sesuai atur lindung anak pondok salafiyah parappe putri ada kegiatan sosialisasi tema cegah tangan keras satu.</v>
+      </c>
+    </row>
+    <row r="1566" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1566" s="2">
         <v>1565</v>
       </c>
@@ -24608,8 +25041,12 @@
       <c r="D1566" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1567" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1566" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>biasax seniorx beri hukum tdk sesuai lindung anak pondok salafiyah parappe putri ada kegiatan sosialisasi tema cegah tangan keras satu.</v>
+      </c>
+    </row>
+    <row r="1567" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1567" s="2">
         <v>1566</v>
       </c>
@@ -24622,8 +25059,12 @@
       <c r="D1567" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1568" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1567" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>aamiin selamat ulang tahun negara cinta tanah air, semoga tetap aman damai limpah barokah.</v>
+      </c>
+    </row>
+    <row r="1568" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1568" s="2">
         <v>1567</v>
       </c>
@@ -24636,8 +25077,12 @@
       <c r="D1568" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1569" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1568" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>aamiin selamat ulang tahun negara cinta tanah air, semoga tetap aman damai limpah barokah.</v>
+      </c>
+    </row>
+    <row r="1569" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1569" s="2">
         <v>1568</v>
       </c>
@@ -24650,8 +25095,12 @@
       <c r="D1569" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1570" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1569" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>hebat selamat ulang tahun negara cinta tanah air, semoga tetap aman damai limpah barokah.</v>
+      </c>
+    </row>
+    <row r="1570" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1570" s="2">
         <v>1569</v>
       </c>
@@ -24664,8 +25113,12 @@
       <c r="D1570" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1571" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1570" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>Masyaallahhh seremonial pembukaan porseni antar alumni salafiyah parappe.</v>
+      </c>
+    </row>
+    <row r="1571" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1571" s="2">
         <v>1570</v>
       </c>
@@ -24678,8 +25131,12 @@
       <c r="D1571" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1572" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1571" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>Sukses selalu untuk pondok pes salafiyah parappe seremonial pembukaan porseni antar alumni.</v>
+      </c>
+    </row>
+    <row r="1572" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1572" s="2">
         <v>1571</v>
       </c>
@@ -24692,8 +25149,12 @@
       <c r="D1572" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1573" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1572" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>amin rabbal alamin seremonial pembukaan porseni antar alumni salafiyah Parappe:.</v>
+      </c>
+    </row>
+    <row r="1573" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1573" s="2">
         <v>1572</v>
       </c>
@@ -24706,8 +25167,12 @@
       <c r="D1573" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1574" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1573" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>Moga allah selalu mendapatkan berkah dan sehat selalu dan sukses selalu untuk anak dan semua alumni pp salapiyah parappe amiin yaa allah seremonial pembukaan porseni antar alumni pp salapiyah parappe.</v>
+      </c>
+    </row>
+    <row r="1574" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1574" s="2">
         <v>1573</v>
       </c>
@@ -24720,8 +25185,12 @@
       <c r="D1574" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1575" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1574" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>masya allah galeri buka porseni antar putri pondok salafiyah parappe putri tema kompak kompetisi bangun karakter islami.</v>
+      </c>
+    </row>
+    <row r="1575" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1575" s="2">
         <v>1574</v>
       </c>
@@ -24734,8 +25203,12 @@
       <c r="D1575" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1576" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1575" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>galeri buka porseni antar putri pondok salafiyah parappe putri tema kompak kompetisi bangun karakter islami.</v>
+      </c>
+    </row>
+    <row r="1576" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1576" s="2">
         <v>1575</v>
       </c>
@@ -24748,8 +25221,12 @@
       <c r="D1576" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1577" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="E1576" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>masya Allah smga sht sllu nak hisra galeri buka porseni antar parappe putri pondok salafiyah tema kompak kompetisi ukiran prestasi bangun karakter islami.</v>
+      </c>
+    </row>
+    <row r="1577" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A1577" s="2">
         <v>1576</v>
       </c>
@@ -24762,8 +25239,12 @@
       <c r="D1577" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1578" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1577" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>Semangat Ana Solehaku tunjjkn kaliapun apresiasi dg mengikuti perkembangan jaman tentu koridor benar galeri buka porseni antar parappe putri pondok salafiyah parappe putri tema kompak kompetisi ukir prestasi bangun karakter islami.</v>
+      </c>
+    </row>
+    <row r="1578" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1578" s="2">
         <v>1577</v>
       </c>
@@ -24776,8 +25257,12 @@
       <c r="D1578" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1579" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1578" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>masya allah sehat selalu nak galeri buka porseni antar parappe putri pondok salafiyah parappe putri tema kompak kompetisi membangun karakter islami.</v>
+      </c>
+    </row>
+    <row r="1579" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1579" s="2">
         <v>1578</v>
       </c>
@@ -24790,8 +25275,12 @@
       <c r="D1579" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1580" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1579" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>aamiin... ...hari-hari yang mulia... ...moga Allah mulia kita di dunia dan di akhirat..</v>
+      </c>
+    </row>
+    <row r="1580" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1580" s="2">
         <v>1579</v>
       </c>
@@ -24804,8 +25293,12 @@
       <c r="D1580" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1581" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1580" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>amiiiinn mulia hari hari mulia, semoga allah mulia dunia akhirat kita,.</v>
+      </c>
+    </row>
+    <row r="1581" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1581" s="2">
         <v>1580</v>
       </c>
@@ -24818,8 +25311,12 @@
       <c r="D1581" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1582" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1581" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>aamiin... ...hari-hari yang mulia... ...moga Allah mulia kita di dunia dan di akhirat..</v>
+      </c>
+    </row>
+    <row r="1582" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1582" s="2">
         <v>1581</v>
       </c>
@@ -24832,8 +25329,12 @@
       <c r="D1582" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1583" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1582" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>aamiin... ...hari-hari yang mulia... ...moga Allah mulia kita di dunia dan di akhirat..</v>
+      </c>
+    </row>
+    <row r="1583" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1583" s="2">
         <v>1582</v>
       </c>
@@ -24846,8 +25347,12 @@
       <c r="D1583" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1584" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1583" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>amin mulia hari hari mulia moga allah mulia dunia akhirat kita.</v>
+      </c>
+    </row>
+    <row r="1584" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1584" s="2">
         <v>1583</v>
       </c>
@@ -24860,8 +25365,12 @@
       <c r="D1584" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1585" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1584" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>aamiiin, hari hari yang mulia, semoga Allah muliakan dunia dan akhirat kita,.</v>
+      </c>
+    </row>
+    <row r="1585" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1585" s="2">
         <v>1584</v>
       </c>
@@ -24874,8 +25383,12 @@
       <c r="D1585" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1586" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1585" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>aamiin... ...hari-hari yang mulia... ...moga Allah mulia kita di dunia dan di akhirat..</v>
+      </c>
+    </row>
+    <row r="1586" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1586" s="2">
         <v>1585</v>
       </c>
@@ -24888,8 +25401,12 @@
       <c r="D1586" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1587" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1586" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>aamiin... ...hari-hari yang mulia... ...moga Allah mulia kita di dunia dan di akhirat..</v>
+      </c>
+    </row>
+    <row r="1587" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1587" s="2">
         <v>1586</v>
       </c>
@@ -24902,8 +25419,12 @@
       <c r="D1587" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1588" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1587" s="5" t="str">
+        <f t="shared" ref="E1587:E1617" si="2">_xlfn.CONCAT(C1587,".")</f>
+        <v>amiin allahhuma amiin mulia hari hari mulia moga allah mulia kita dengan baik dunia dan akhirat.</v>
+      </c>
+    </row>
+    <row r="1588" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1588" s="2">
         <v>1587</v>
       </c>
@@ -24916,8 +25437,12 @@
       <c r="D1588" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1589" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1588" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>aaaaaamin mulia hari hari mulia, semoga Allah mulia kita di dunia dan di akhirat,.</v>
+      </c>
+    </row>
+    <row r="1589" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1589" s="2">
         <v>1588</v>
       </c>
@@ -24930,8 +25455,12 @@
       <c r="D1589" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1590" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1589" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>aamiin robbal alamin mulia hari hari mulia, semoga allah mulia kita di dunia dan akhirat,.</v>
+      </c>
+    </row>
+    <row r="1590" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1590" s="2">
         <v>1589</v>
       </c>
@@ -24944,8 +25473,12 @@
       <c r="D1590" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1591" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1590" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>aamiin allahhumma aamiin mulia hari hari mulia moga allah mulia dunia akhirat kita.</v>
+      </c>
+    </row>
+    <row r="1591" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1591" s="2">
         <v>1590</v>
       </c>
@@ -24958,8 +25491,12 @@
       <c r="D1591" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1592" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1591" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>aamiiin moment haru pisah dari salah satu asaidzah pondok salafiyah parappe putri ustadzah nur hidayah syahdan tempat tugas baru nya.</v>
+      </c>
+    </row>
+    <row r="1592" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1592" s="2">
         <v>1591</v>
       </c>
@@ -24972,8 +25509,12 @@
       <c r="D1592" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1593" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1592" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>aamiin moment haru pisah dari salah satu asaidzah pondok salafiyah parappe putri ustadzah nur hidayah syahdan tempat tugas baru nya.</v>
+      </c>
+    </row>
+    <row r="1593" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1593" s="2">
         <v>1592</v>
       </c>
@@ -24986,8 +25527,12 @@
       <c r="D1593" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1594" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1593" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>asmin yra moment haru berpisah salah satu asaidzah pondok salafiyah parappe putri ustadzah nur hidayah syahdan tempat tugas baru nya.</v>
+      </c>
+    </row>
+    <row r="1594" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1594" s="2">
         <v>1593</v>
       </c>
@@ -25000,8 +25545,12 @@
       <c r="D1594" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1595" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1594" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>Moga sehat selalu d tempt baru ustzah hidayah aamiin moment haru pisah salah satu asaidzah pondok salafiyah parappe putri ustadzah nur hidayah syahdan tempat tugas baru nya.</v>
+      </c>
+    </row>
+    <row r="1595" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1595" s="2">
         <v>1594</v>
       </c>
@@ -25014,8 +25563,12 @@
       <c r="D1595" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1596" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1595" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>amiin yra moment haru berpisah salah satu asaidzah pondok salafiyah parappe putri ustadzah nur hidayah syahdan tempat tugas baru nya.</v>
+      </c>
+    </row>
+    <row r="1596" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1596" s="2">
         <v>1595</v>
       </c>
@@ -25028,8 +25581,12 @@
       <c r="D1596" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1597" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1596" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>kak hikmaa sehat selalu tempat baruta ustadzah moment haru pisah salah satu asaidzah pondok salafiyah parappe putri ustadzah nur hidayah syahdan tempat tugas baru nya.</v>
+      </c>
+    </row>
+    <row r="1597" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1597" s="2">
         <v>1596</v>
       </c>
@@ -25042,8 +25599,12 @@
       <c r="D1597" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1598" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1597" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>masya allah galeri ta aruf dibuka untuk parappe putri, parappe putri dari pondok salafiyah.</v>
+      </c>
+    </row>
+    <row r="1598" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1598" s="2">
         <v>1597</v>
       </c>
@@ -25056,8 +25617,12 @@
       <c r="D1598" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1599" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1598" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>Sehat sll semua Galeri Buka Ta Aruf Santriwati Baru di Ponpes Salafiyah Parappe Putri.</v>
+      </c>
+    </row>
+    <row r="1599" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1599" s="2">
         <v>1598</v>
       </c>
@@ -25070,8 +25635,12 @@
       <c r="D1599" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1600" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1599" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>mas syaa allaah sehatki semua nak antara adam putri alhamdulillah galeri buka ta aruf parappe putri baru.</v>
+      </c>
+    </row>
+    <row r="1600" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1600" s="2">
         <v>1599</v>
       </c>
@@ -25084,8 +25653,12 @@
       <c r="D1600" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1601" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1600" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>mantap smg parappe putri semakin majuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuu.</v>
+      </c>
+    </row>
+    <row r="1601" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1601" s="2">
         <v>1600</v>
       </c>
@@ -25098,8 +25671,12 @@
       <c r="D1601" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1602" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1601" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>Tabarakallah Sehat Semua Galeri Buka Ta Aruf Santriwati Baru di Ponpes Salafiyah Parappe Putri.</v>
+      </c>
+    </row>
+    <row r="1602" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1602" s="2">
         <v>1601</v>
       </c>
@@ -25112,8 +25689,12 @@
       <c r="D1602" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1603" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1602" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>luar biasa xd ada dokumentasi hari berikutnya galeri buka ta aruf, parappe putri, seorang putri dari pondok salafiyah.</v>
+      </c>
+    </row>
+    <row r="1603" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1603" s="2">
         <v>1602</v>
       </c>
@@ -25126,8 +25707,12 @@
       <c r="D1603" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1604" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1603" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>Ta Aruf Galeri Buka Ta Aruf Santriwati Baru di Ponpes Salafiyah Parappe Putri.</v>
+      </c>
+    </row>
+    <row r="1604" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1604" s="2">
         <v>1603</v>
       </c>
@@ -25140,8 +25725,12 @@
       <c r="D1604" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1605" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1604" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>alhamdulillah sehatki semua nak antara adam putri galeri buka ta aruf, parappe putri,.</v>
+      </c>
+    </row>
+    <row r="1605" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1605" s="2">
         <v>1604</v>
       </c>
@@ -25154,8 +25743,12 @@
       <c r="D1605" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1606" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1605" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>masya allah sehatji semua nak antara ada putri galeri buka ta aruf putri baru dari pondok salafiyah parappe putri.</v>
+      </c>
+    </row>
+    <row r="1606" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1606" s="2">
         <v>1605</v>
       </c>
@@ -25168,8 +25761,12 @@
       <c r="D1606" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1607" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1606" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>masya allah ankku tidak kliatan galeri buka ta aruf parappe putri.</v>
+      </c>
+    </row>
+    <row r="1607" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1607" s="2">
         <v>1606</v>
       </c>
@@ -25182,8 +25779,12 @@
       <c r="D1607" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1608" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1607" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>masya allah anak syaleha semua moga dpt menjadi cermin bagi adik adikx musyawarah kitab fathul qorib fathul mu in pdf ulya pdf wustho.</v>
+      </c>
+    </row>
+    <row r="1608" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1608" s="2">
         <v>1607</v>
       </c>
@@ -25196,8 +25797,12 @@
       <c r="D1608" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1609" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1608" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>masya allah musyawarah kitab fathul qarib antar para ulama thobaqoh fathul qorib fathul mu in pdf ulya pdf wustho.</v>
+      </c>
+    </row>
+    <row r="1609" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1609" s="2">
         <v>1608</v>
       </c>
@@ -25210,8 +25815,12 @@
       <c r="D1609" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1610" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1609" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>masya allah moga anak anak juga seperti musyawarah kitab fathul qorib fathul mu in pdf ulya pdf wustho.</v>
+      </c>
+    </row>
+    <row r="1610" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1610" s="2">
         <v>1609</v>
       </c>
@@ -25224,8 +25833,12 @@
       <c r="D1610" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1611" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1610" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>Tetap semangat anakku, moga sukses musyawarah kitab fathul qarib antar alumni thobaqoh fathul qorib fathul mu in pdf ulya pdf wustho.</v>
+      </c>
+    </row>
+    <row r="1611" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1611" s="2">
         <v>1610</v>
       </c>
@@ -25238,8 +25851,12 @@
       <c r="D1611" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1612" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E1611" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>masyaallah semangat anak, semoga ilmunya berkah musyawarah kitab fathul qarib antar para ulama thobaqoh fathul qorib fathul mu in pdf ulya pdf wustho.</v>
+      </c>
+    </row>
+    <row r="1612" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1612" s="2">
         <v>1611</v>
       </c>
@@ -25252,8 +25869,12 @@
       <c r="D1612" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1613" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1612" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>ingat jaman dulu ketika mas d polmas musyawarah kitab fathul qarib antar satriwati thobaqoh fathul qorib fathul mu in pdf ulya pdf wustho.</v>
+      </c>
+    </row>
+    <row r="1613" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1613" s="2">
         <v>1612</v>
       </c>
@@ -25266,8 +25887,12 @@
       <c r="D1613" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1614" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1613" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>Buka Pendaftaran Santriwati Baru di Ponpes Salafiyah Parappe.</v>
+      </c>
+    </row>
+    <row r="1614" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1614" s="2">
         <v>1613</v>
       </c>
@@ -25280,8 +25905,12 @@
       <c r="D1614" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1615" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1614" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>Bisa Share Buka Pendaftaran Santriwati Baru di Ponpes Salafiyah Parappe.</v>
+      </c>
+    </row>
+    <row r="1615" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1615" s="2">
         <v>1614</v>
       </c>
@@ -25294,8 +25923,12 @@
       <c r="D1615" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1616" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1615" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>iya bisa share buka daftar calon siswa salafiiyah parappe.</v>
+      </c>
+    </row>
+    <row r="1616" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1616" s="2">
         <v>1615</v>
       </c>
@@ -25308,8 +25941,12 @@
       <c r="D1616" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1617" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1616" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>insyaallah tahun anak-anak dibuka pendaftaran calon siswa baru di pondok salafiyah parappe.</v>
+      </c>
+    </row>
+    <row r="1617" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1617" s="2">
         <v>1616</v>
       </c>
@@ -25321,6 +25958,10 @@
       </c>
       <c r="D1617" s="3" t="s">
         <v>6</v>
+      </c>
+      <c r="E1617" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>Keren membuka daftar baru Santriwati di Ponpes Salafiyah Parappe.</v>
       </c>
     </row>
   </sheetData>

</xml_diff>